<commit_message>
feat(template): restyle ABC template to match variance visual language
Header row now uses FFF2F2F2 gray with thin borders, center/middle,
size 11 — identical to the variance analysis template. Added navy
title bar (row 1) and light slate instructions row (row 2), freeze
pane at row 4, autofilter on headers, and proper column widths.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/template-abc.xlsx
+++ b/public/template-abc.xlsx
@@ -1,58 +1,117 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Template" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Dati ABC" state="visible" r:id="rId4"/>
   </sheets>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="11">
+  <si>
+    <t>Template Matrice ABC — MarginView</t>
+  </si>
+  <si>
+    <t>Colonne obbligatorie: Articolo, Fatturato, Categoria, Margine %. Opzionali: Brand, Costo del Venduto, Giacenza di Magazzino (€).</t>
+  </si>
+  <si>
+    <t>Articolo</t>
+  </si>
+  <si>
+    <t>Descrizione</t>
+  </si>
+  <si>
+    <t>Brand</t>
+  </si>
+  <si>
+    <t>Categoria</t>
+  </si>
+  <si>
+    <t>Fatturato</t>
+  </si>
+  <si>
+    <t>Costo del Venduto</t>
+  </si>
+  <si>
+    <t>Margine %</t>
+  </si>
+  <si>
+    <t>Giacenza di Magazzino (€)</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+    <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="12"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <i/>
+      <color rgb="FF64748B"/>
+      <sz val="9"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1E2761"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF1F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8FAFC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -60,18 +119,65 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFCBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="10">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="3" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="3" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,58 +502,207 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="20.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="32" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="19" customWidth="1"/>
+    <col min="7" max="7" width="13" customWidth="1"/>
+    <col min="8" max="8" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Template Matrice ABC — MarginView</v>
-      </c>
+    <row r="1" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Colonne obbligatorie: Articolo, Fatturato, Categoria, Margine (%). Opzionali: Brand, Costo del Venduto, Giacenza di Magazzino (€).</v>
-      </c>
+    <row r="2" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Articolo</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Descrizione</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Brand</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Categoria</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Fatturato</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Costo del Venduto</v>
-      </c>
-      <c r="G3" t="str">
-        <v>Margine %</v>
-      </c>
-      <c r="H3" t="str">
-        <v>Giacenza di Magazzino (€)</v>
+    <row r="3" ht="25" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
-  </ignoredErrors>
+  <autoFilter ref="A3:H3"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>